<commit_message>
Kapitola 8: opravy po odborné a didaktické revizi
</commit_message>
<xml_diff>
--- a/data/kapitola_08.xlsx
+++ b/data/kapitola_08.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C2F63D0-0742-4199-9D9A-B8D7B7F81AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5928BB13-6C8B-4929-9FFD-15FE4BCBFF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{D0A71B8E-9AED-4BA1-8D1D-236B42023A54}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{D5808EF5-B59F-4B16-A6A8-FA3446190DDF}"/>
   </bookViews>
   <sheets>
     <sheet name="Prehled" sheetId="1" r:id="rId1"/>
@@ -409,7 +409,7 @@
     <t>Směrodatná odchylka hmotnosti před terapií (kg)</t>
   </si>
   <si>
-    <t>Výklad: měření před a po bez kontrolní skupiny; volba směrodatné odchylky pro d</t>
+    <t>Párová analýza skupiny s terapií; porovnání s kontrolou není součástí výpočtu.</t>
   </si>
   <si>
     <t>Skutečná data: Everitt podle Howella (2013, tab. 7.3, s. 198–199). Howell uvádí libry; souhrny byly spočítány z hodnot převedených na kilogramy (1 lb = 0,45359237 kg) a zaokrouhleny na tři desetinná místa. Jednotlivé hodnoty sešit neobsahuje.</t>
@@ -1211,7 +1211,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73E2853A-BE4B-4509-9D5B-4709D32AE0CD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBFA3B1D-DCAD-4F04-B17C-7416B7F2BA44}">
   <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1507,7 +1507,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{508932FB-BD3A-48F1-88EA-8BB50946D6D9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A274334-6DAA-4E46-BFF1-52175C059F7F}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1595,7 +1595,7 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4145E816-F557-45AA-9D78-8483ADECC528}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358D37EE-6B05-4778-91B3-3D4A720C72A2}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1677,7 +1677,7 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87E191AE-4CA0-46AA-8BA1-F6F32ECBA6E2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EF4E61B-4CD7-4BBA-B089-F8841FC86331}">
   <dimension ref="A1:F33"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2170,7 +2170,7 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A130E4C9-7EAF-480A-9337-38BC79E72E26}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBAD7620-F54E-433E-82F2-B49CA56FABC5}">
   <dimension ref="A1:G7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2260,7 +2260,7 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{257C73B1-92D1-444B-A815-6796CA49E90A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CDAE2E9-1943-4E24-A3A7-911CDB0A1495}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2330,7 +2330,7 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{939F796E-B00A-4FB8-8536-A423A51C0845}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C25E36B8-FDE6-4838-AF60-9A79E8113E76}">
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2533,7 +2533,7 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC0F457B-AA4F-4A17-95A7-95874AAD5D93}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{538E06F6-6FDF-455A-95B0-2DAA270AB3AD}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2615,7 +2615,7 @@
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB6B5DF0-B1B4-40DB-A96D-93F777F52063}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D05483C2-8AB4-4084-90D9-6C45E7E7EB16}">
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2824,7 +2824,7 @@
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45A4E35D-3013-458C-9264-85582F604E22}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00873DA0-EBB8-4CE9-AD60-1F06D8E1D56A}">
   <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2906,7 +2906,7 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28EFB8D0-84D4-4759-AE57-E0667F47AC34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B08393-1433-4F1F-8003-712DB1AF171C}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2988,7 +2988,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34F453E9-F368-4D18-B2E8-5AC1F8FD8A48}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAEBA6EF-5F9A-43E2-9F70-B61474B8C90D}">
   <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3607,7 +3607,7 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{972C4357-4CF5-4362-AAE6-82C780A20675}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BD417C3-B0C0-4126-830F-3D7F6228165C}">
   <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3703,7 +3703,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AAE3D61-4C19-4935-84A2-D75E26A5B310}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CBACE6C-A3BA-408F-A6BB-0D20F5624333}">
   <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4177,7 +4177,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5C722B5-4BA7-402B-83B4-FCEE23DEABF6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2771DAD3-2B2C-4DC7-B1A4-9536279F4000}">
   <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4654,7 +4654,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD90DCF5-EE5C-414D-8383-942E93103657}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF6A7750-F40F-4BBD-AF4D-02DFC62B0259}">
   <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5338,7 +5338,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA1F06DE-106E-4BAF-BA9A-3EE0B00EF9F4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{245F1995-01C9-470E-976B-381BF48599B6}">
   <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5855,7 +5855,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EB776A9-5829-498D-8DFB-E71675B53019}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A03C3FE4-F7DB-4F3D-8BA7-9610862618A3}">
   <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6038,7 +6038,7 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2DB608F-F74A-41A2-8E90-58A21A091F67}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4977FBF0-420B-47A0-9194-B326F3349089}">
   <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6281,7 +6281,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB2A2A4F-77EE-4C31-8AD6-682345D3D837}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{864861A8-43C9-4D70-933A-7EF3CD3D4888}">
   <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>